<commit_message>
Creacion Index - IceDux
</commit_message>
<xml_diff>
--- a/ES/Datos/A8/Aire_du_Reyran_A8_Public_Reviews_Analysis.xlsx
+++ b/ES/Datos/A8/Aire_du_Reyran_A8_Public_Reviews_Analysis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nube\iCloudDrive\Trabajo\GitHub\aires-pl-a7-a8-a9\ES\Datos\A8\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{35664631-4762-48E2-9A82-D900AAC66FBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE9B0C92-8911-40B1-B7FB-97508D9D4643}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6DBB6517-C467-4FAD-8182-EC50ED908EFB}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="187">
   <si>
     <t>Autopista</t>
   </si>
@@ -94,9 +94,6 @@
   </si>
   <si>
     <t>https://maps.app.goo.gl/hMnNqnjvhyyvhZ4r7</t>
-  </si>
-  <si>
-    <t>resena</t>
   </si>
   <si>
     <t>jogras mj</t>
@@ -158,9 +155,6 @@
   </si>
   <si>
     <t>Me robaron unos 500 litros de combustible durante la noche del 26 al 27 de febrero de 2026. El aparcamiento estaba iluminado, pero aun así ocurrió. Aparqué en la zona del árbol de Navidad; había un sitio libre a la izquierda y por ahí me sacaron el gasoil. No oí nada porque estaba dormido. Hicieron un trabajo profesional: no me di cuenta de nada durante la inspección matutina del camión, sino más tarde, después de rodar un poco. Incluso volvieron a poner el tapón de goma del depósito; no tenían ninguna prisa. ¡Mucha suerte a todos y tengan mucho cuidado en este aparcamiento!</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/reviews/data=!4m8!14m7!1m6!2m5!1sCi9DQUlRQUNvZENodHljRjlvT2tSWFFsVnRYMmhRWW1kaVR6WmpMVWRpTURKSE1XYxAB!2m1!1s0x0:0x32b0efb1133d59a!3m1!1s2@1:CAIQACodChtycF9oOkRXQlVtX2hQYmdiTzZjLUdiMDJHMWc%7C%7C</t>
   </si>
   <si>
     <t>Hola, Gracias por sus comentarios. Su seguridad en nuestras áreas de descanso es nuestra prioridad, por lo que condenamos enérgicamente estas acciones. Nuestros equipos están colaborando estrechamente con las autoridades para abordar este problema. Le animamos a que les avise llamando al 112. Esperamos que sus próximos viajes transcurran sin incidentes. Solène, Servicio de Atención al Cliente de VINCI Autoroutes</t>
@@ -541,6 +535,115 @@
   <si>
     <t>Po</t>
   </si>
+  <si>
+    <t>AUD-A8-REYRAN-01</t>
+  </si>
+  <si>
+    <t>Respuesta del propietario Hace 8 meses
+Hola,
+Gracias por su mensaje. Su seguridad es nuestra máxima prioridad y condenamos enérgicamente este tipo de comportamiento. Nuestros equipos permanecen movilizados junto con las fuerzas del orden para garantizar un entorno seguro. Por lo tanto, les hemos remitido su informe. Le animamos a que también denuncie cualquier comportamiento sospechoso a la policía llamando al 112.
+Esperamos que sus próximos viajes sean lo más tranquilos posible.
+Solène, Servicio de Atención al Cliente de VINCI Autoroutes</t>
+  </si>
+  <si>
+    <t>AUD-A8-REYRAN-0002</t>
+  </si>
+  <si>
+    <t>AUD-A8-REYRAN-0003</t>
+  </si>
+  <si>
+    <t>AUD-A8-REYRAN-0004</t>
+  </si>
+  <si>
+    <t>AUD-A8-REYRAN-0005</t>
+  </si>
+  <si>
+    <t>AUD-A8-REYRAN-0006</t>
+  </si>
+  <si>
+    <t>https://maps.app.goo.gl/XNWaCXiWUxJJD22HA</t>
+  </si>
+  <si>
+    <t>AUD-A8-REYRAN-0007</t>
+  </si>
+  <si>
+    <t>AUD-A8-REYRAN-0008</t>
+  </si>
+  <si>
+    <t>AUD-A8-REYRAN-0009</t>
+  </si>
+  <si>
+    <t>AUD-A8-REYRAN-0010</t>
+  </si>
+  <si>
+    <t>AUD-A8-REYRAN-0011</t>
+  </si>
+  <si>
+    <t>AUD-A8-REYRAN-0012</t>
+  </si>
+  <si>
+    <t>AUD-A8-REYRAN-0013</t>
+  </si>
+  <si>
+    <t>AUD-A8-REYRAN-0014</t>
+  </si>
+  <si>
+    <t>AUD-A8-REYRAN-0015</t>
+  </si>
+  <si>
+    <t>AUD-A8-REYRAN-0016</t>
+  </si>
+  <si>
+    <t>AUD-A8-REYRAN-0017</t>
+  </si>
+  <si>
+    <t>AUD-A8-REYRAN-0018</t>
+  </si>
+  <si>
+    <t>AUD-A8-REYRAN-0019</t>
+  </si>
+  <si>
+    <t>AUD-A8-REYRAN-0020</t>
+  </si>
+  <si>
+    <t>AUD-A8-REYRAN-0021</t>
+  </si>
+  <si>
+    <t>AUD-A8-REYRAN-0024</t>
+  </si>
+  <si>
+    <t>AUD-A8-REYRAN-0023</t>
+  </si>
+  <si>
+    <t>AUD-A8-REYRAN-0022</t>
+  </si>
+  <si>
+    <t>AUD-A8-REYRAN-0025</t>
+  </si>
+  <si>
+    <t>AUD-A8-REYRAN-0026</t>
+  </si>
+  <si>
+    <t>AUD-A8-REYRAN-0027</t>
+  </si>
+  <si>
+    <t>AUD-A8-REYRAN-0028</t>
+  </si>
+  <si>
+    <t>AUD-A8-REYRAN-0029</t>
+  </si>
+  <si>
+    <t>AUD-A8-REYRAN-0030</t>
+  </si>
+  <si>
+    <t>AUD-A8-REYRAN-0031</t>
+  </si>
+  <si>
+    <t>AUD-A8-REYRAN-0032</t>
+  </si>
+  <si>
+    <t>AUD-A8-REYRAN-0033</t>
+  </si>
 </sst>
 </file>
 
@@ -549,7 +652,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;MAPS-&quot;000"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -638,14 +741,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="204"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -754,21 +849,18 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="6">
+  <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -788,7 +880,7 @@
     <xf numFmtId="164" fontId="5" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="5" applyFill="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="4" applyFill="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="11" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -818,31 +910,28 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="1" xfId="4" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="14" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="13" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -854,6 +943,12 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="3">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="4">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -861,12 +956,11 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="5">
     <cellStyle name="20% - Énfasis1" xfId="1" builtinId="30"/>
     <cellStyle name="60% - Énfasis5" xfId="2" builtinId="48"/>
-    <cellStyle name="Autopista" xfId="5" xr:uid="{EB88B4C3-1DAA-4445-9EE1-456C100FD6D1}"/>
+    <cellStyle name="Autopista" xfId="4" xr:uid="{EB88B4C3-1DAA-4445-9EE1-456C100FD6D1}"/>
     <cellStyle name="Hipervínculo" xfId="3" builtinId="8"/>
-    <cellStyle name="Hipervínculo visitado" xfId="4" builtinId="9"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1270,60 +1364,59 @@
   <dimension ref="A1:J38"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.42578125" style="19" customWidth="1"/>
+    <col min="1" max="1" width="25.28515625" style="18" customWidth="1"/>
     <col min="2" max="2" width="20.42578125" style="5" customWidth="1"/>
     <col min="3" max="3" width="21.28515625" style="5" customWidth="1"/>
-    <col min="4" max="4" width="34" style="19" customWidth="1"/>
-    <col min="5" max="5" width="24" style="19" customWidth="1"/>
-    <col min="6" max="6" width="27.42578125" style="19" customWidth="1"/>
-    <col min="7" max="7" width="12" style="19" customWidth="1"/>
-    <col min="8" max="8" width="62" style="24" customWidth="1"/>
-    <col min="9" max="9" width="36" style="19" customWidth="1"/>
+    <col min="4" max="4" width="34" style="18" customWidth="1"/>
+    <col min="5" max="5" width="24" style="18" customWidth="1"/>
+    <col min="6" max="6" width="27.42578125" style="18" customWidth="1"/>
+    <col min="7" max="7" width="12" style="18" customWidth="1"/>
+    <col min="8" max="8" width="62" style="23" customWidth="1"/>
+    <col min="9" max="9" width="36" style="18" customWidth="1"/>
     <col min="10" max="10" width="50.7109375" style="5" customWidth="1"/>
     <col min="11" max="11" width="9.140625" style="5" customWidth="1"/>
     <col min="12" max="16384" width="9.140625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="30" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="1:10" s="30" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="3" spans="1:10" s="30" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="4" spans="1:10" s="29" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="5" spans="1:10" s="28" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="26" t="s">
-        <v>153</v>
-      </c>
-      <c r="B5" s="26" t="s">
-        <v>104</v>
-      </c>
-      <c r="C5" s="26" t="s">
+    <row r="1" spans="1:10" s="31" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:10" s="31" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:10" s="31" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="4" spans="1:10" s="30" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="1:10" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="25" t="s">
+        <v>151</v>
+      </c>
+      <c r="B5" s="25" t="s">
+        <v>102</v>
+      </c>
+      <c r="C5" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="D5" s="26" t="s">
+      <c r="D5" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="E5" s="26" t="s">
+      <c r="E5" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="F5" s="26" t="s">
+      <c r="F5" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="26" t="s">
+      <c r="G5" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="H5" s="27" t="s">
+      <c r="H5" s="26" t="s">
         <v>5</v>
       </c>
-      <c r="I5" s="26" t="s">
+      <c r="I5" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="J5" s="26" t="s">
+      <c r="J5" s="25" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A6" s="6">
-        <f>ROW()-5</f>
-        <v>1</v>
+    <row r="6" spans="1:10" ht="225" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
+        <v>152</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>12</v>
@@ -1350,13 +1443,12 @@
         <v>16</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>17</v>
+        <v>153</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="180" x14ac:dyDescent="0.25">
-      <c r="A7" s="6">
-        <f>ROW()-5</f>
-        <v>2</v>
+      <c r="A7" s="6" t="s">
+        <v>154</v>
       </c>
       <c r="B7" s="7" t="s">
         <v>12</v>
@@ -1368,28 +1460,27 @@
         <v>9</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>13</v>
       </c>
       <c r="G7" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H7" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="H7" s="8" t="s">
+      <c r="I7" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I7" s="2" t="s">
+      <c r="J7" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="J7" s="3" t="s">
-        <v>22</v>
-      </c>
     </row>
     <row r="8" spans="1:10" ht="210" x14ac:dyDescent="0.25">
-      <c r="A8" s="6">
-        <f t="shared" ref="A8:A38" si="0">ROW()-5</f>
-        <v>3</v>
+      <c r="A8" s="6" t="s">
+        <v>155</v>
       </c>
       <c r="B8" s="7" t="s">
         <v>12</v>
@@ -1401,28 +1492,27 @@
         <v>9</v>
       </c>
       <c r="E8" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>24</v>
       </c>
       <c r="G8" s="1" t="s">
         <v>14</v>
       </c>
       <c r="H8" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I8" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="I8" s="10" t="s">
+      <c r="J8" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="J8" s="3" t="s">
-        <v>27</v>
-      </c>
     </row>
     <row r="9" spans="1:10" ht="100.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="6">
-        <f t="shared" si="0"/>
-        <v>4</v>
+      <c r="A9" s="6" t="s">
+        <v>156</v>
       </c>
       <c r="B9" s="7" t="s">
         <v>12</v>
@@ -1434,28 +1524,27 @@
         <v>9</v>
       </c>
       <c r="E9" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>28</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>29</v>
       </c>
       <c r="G9" s="1" t="s">
         <v>14</v>
       </c>
       <c r="H9" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="I9" s="28" t="s">
         <v>30</v>
       </c>
-      <c r="I9" s="2" t="s">
+      <c r="J9" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="J9" s="11" t="s">
-        <v>32</v>
-      </c>
     </row>
     <row r="10" spans="1:10" ht="157.5" x14ac:dyDescent="0.25">
-      <c r="A10" s="6">
-        <f t="shared" si="0"/>
-        <v>5</v>
+      <c r="A10" s="6" t="s">
+        <v>157</v>
       </c>
       <c r="B10" s="7" t="s">
         <v>12</v>
@@ -1467,28 +1556,27 @@
         <v>9</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>13</v>
       </c>
       <c r="G10" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="H10" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="H10" s="8" t="s">
+      <c r="I10" s="28" t="s">
+        <v>159</v>
+      </c>
+      <c r="J10" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="I10" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="J10" s="4" t="s">
-        <v>37</v>
-      </c>
     </row>
     <row r="11" spans="1:10" ht="142.5" x14ac:dyDescent="0.25">
-      <c r="A11" s="6">
-        <f t="shared" si="0"/>
-        <v>6</v>
+      <c r="A11" s="6" t="s">
+        <v>158</v>
       </c>
       <c r="B11" s="7" t="s">
         <v>12</v>
@@ -1500,61 +1588,59 @@
         <v>9</v>
       </c>
       <c r="E11" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="H11" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="I11" s="28" t="s">
         <v>39</v>
       </c>
-      <c r="G11" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="H11" s="8" t="s">
+      <c r="J11" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="I11" s="10" t="s">
+    </row>
+    <row r="12" spans="1:10" ht="171" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="B12" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="J11" s="4" t="s">
+      <c r="C12" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E12" s="10" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="12" spans="1:10" ht="171" x14ac:dyDescent="0.25">
-      <c r="A12" s="6">
-        <f t="shared" si="0"/>
-        <v>7</v>
-      </c>
-      <c r="B12" s="7" t="s">
+      <c r="F12" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C12" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E12" s="10" t="s">
+      <c r="G12" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="H12" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="G12" s="1" t="s">
+      <c r="I12" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="H12" s="8" t="s">
+      <c r="J12" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="I12" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="J12" s="4" t="s">
-        <v>49</v>
-      </c>
     </row>
     <row r="13" spans="1:10" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="6">
-        <f t="shared" si="0"/>
-        <v>8</v>
+      <c r="A13" s="6" t="s">
+        <v>161</v>
       </c>
       <c r="B13" s="7" t="s">
         <v>12</v>
@@ -1566,24 +1652,25 @@
         <v>9</v>
       </c>
       <c r="E13" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="H13" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="I13" s="28" t="s">
         <v>50</v>
       </c>
-      <c r="F13" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="G13" s="1"/>
-      <c r="H13" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="I13" s="2" t="s">
-        <v>52</v>
-      </c>
       <c r="J13" s="4"/>
     </row>
     <row r="14" spans="1:10" ht="180" x14ac:dyDescent="0.25">
-      <c r="A14" s="6">
-        <f t="shared" si="0"/>
-        <v>9</v>
+      <c r="A14" s="6" t="s">
+        <v>162</v>
       </c>
       <c r="B14" s="7" t="s">
         <v>12</v>
@@ -1595,61 +1682,59 @@
         <v>9</v>
       </c>
       <c r="E14" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H14" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="I14" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="F14" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="H14" s="8" t="s">
+      <c r="J14" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="I14" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="J14" s="3" t="s">
-        <v>56</v>
-      </c>
     </row>
     <row r="15" spans="1:10" s="16" customFormat="1" ht="165" x14ac:dyDescent="0.25">
-      <c r="A15" s="6">
-        <f t="shared" si="0"/>
-        <v>10</v>
+      <c r="A15" s="6" t="s">
+        <v>163</v>
       </c>
       <c r="B15" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C15" s="13" t="s">
+      <c r="C15" s="29" t="s">
         <v>8</v>
       </c>
       <c r="D15" s="13" t="s">
         <v>9</v>
       </c>
       <c r="E15" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="F15" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="G15" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="H15" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="I15" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="F15" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="G15" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="H15" s="14" t="s">
+      <c r="J15" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="I15" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="J15" s="15" t="s">
-        <v>60</v>
-      </c>
     </row>
     <row r="16" spans="1:10" s="16" customFormat="1" ht="165" x14ac:dyDescent="0.25">
-      <c r="A16" s="6">
-        <f t="shared" si="0"/>
-        <v>11</v>
+      <c r="A16" s="6" t="s">
+        <v>164</v>
       </c>
       <c r="B16" s="7" t="s">
         <v>12</v>
@@ -1660,60 +1745,58 @@
       <c r="D16" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="E16" s="17" t="s">
+      <c r="E16" s="28" t="s">
+        <v>59</v>
+      </c>
+      <c r="F16" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="G16" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="F16" s="13" t="s">
+      <c r="H16" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="G16" s="13" t="s">
+      <c r="I16" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="H16" s="14" t="s">
+      <c r="J16" s="15" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E17" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="I16" s="10" t="s">
+      <c r="F17" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H17" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="J16" s="15" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A17" s="6">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="B17" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="C17" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E17" s="10" t="s">
+      <c r="I17" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="F17" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="H17" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="I17" s="9" t="s">
-        <v>68</v>
-      </c>
       <c r="J17" s="3"/>
     </row>
     <row r="18" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A18" s="6">
-        <f t="shared" si="0"/>
-        <v>13</v>
+      <c r="A18" s="6" t="s">
+        <v>166</v>
       </c>
       <c r="B18" s="7" t="s">
         <v>12</v>
@@ -1725,28 +1808,27 @@
         <v>9</v>
       </c>
       <c r="E18" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="G18" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="H18" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="G18" s="1" t="s">
+      <c r="I18" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="H18" s="8" t="s">
+      <c r="J18" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="I18" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="J18" s="18" t="s">
-        <v>74</v>
-      </c>
     </row>
     <row r="19" spans="1:10" ht="21" x14ac:dyDescent="0.25">
-      <c r="A19" s="6">
-        <f t="shared" si="0"/>
-        <v>14</v>
+      <c r="A19" s="6" t="s">
+        <v>167</v>
       </c>
       <c r="B19" s="7"/>
       <c r="C19" s="7"/>
@@ -1759,9 +1841,8 @@
       <c r="J19" s="3"/>
     </row>
     <row r="20" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A20" s="6">
-        <f t="shared" si="0"/>
-        <v>15</v>
+      <c r="A20" s="6" t="s">
+        <v>168</v>
       </c>
       <c r="B20" s="7" t="s">
         <v>12</v>
@@ -1773,28 +1854,27 @@
         <v>9</v>
       </c>
       <c r="E20" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="G20" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="F20" s="1" t="s">
+      <c r="H20" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="I20" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="G20" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="H20" s="8" t="s">
+      <c r="J20" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="I20" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="J20" s="18" t="s">
-        <v>74</v>
-      </c>
     </row>
     <row r="21" spans="1:10" ht="63" x14ac:dyDescent="0.25">
-      <c r="A21" s="6">
-        <f t="shared" si="0"/>
-        <v>16</v>
+      <c r="A21" s="6" t="s">
+        <v>169</v>
       </c>
       <c r="B21" s="7" t="s">
         <v>12</v>
@@ -1806,26 +1886,25 @@
         <v>9</v>
       </c>
       <c r="E21" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="H21" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="F21" s="1" t="s">
+      <c r="I21" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="G21" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="H21" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="I21" s="2" t="s">
-        <v>82</v>
-      </c>
       <c r="J21" s="3"/>
     </row>
     <row r="22" spans="1:10" ht="82.5" x14ac:dyDescent="0.25">
-      <c r="A22" s="6">
-        <f t="shared" si="0"/>
-        <v>17</v>
+      <c r="A22" s="6" t="s">
+        <v>170</v>
       </c>
       <c r="B22" s="7" t="s">
         <v>12</v>
@@ -1837,25 +1916,24 @@
         <v>9</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="F22" s="19" t="s">
-        <v>70</v>
-      </c>
-      <c r="G22" s="19" t="s">
-        <v>86</v>
-      </c>
-      <c r="H22" s="20" t="s">
         <v>83</v>
       </c>
+      <c r="F22" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="G22" s="18" t="s">
+        <v>84</v>
+      </c>
+      <c r="H22" s="19" t="s">
+        <v>81</v>
+      </c>
       <c r="I22" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="90" x14ac:dyDescent="0.25">
-      <c r="A23" s="6">
-        <f t="shared" si="0"/>
-        <v>18</v>
+      <c r="A23" s="6" t="s">
+        <v>171</v>
       </c>
       <c r="B23" s="7" t="s">
         <v>12</v>
@@ -1867,25 +1945,24 @@
         <v>9</v>
       </c>
       <c r="E23" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="F23" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="G23" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="H23" s="20" t="s">
         <v>87</v>
       </c>
-      <c r="F23" s="19" t="s">
-        <v>70</v>
-      </c>
-      <c r="G23" s="19" t="s">
-        <v>77</v>
-      </c>
-      <c r="H23" s="21" t="s">
-        <v>89</v>
-      </c>
       <c r="I23" s="2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="75" x14ac:dyDescent="0.25">
-      <c r="A24" s="6">
-        <f t="shared" si="0"/>
-        <v>19</v>
+      <c r="A24" s="6" t="s">
+        <v>172</v>
       </c>
       <c r="B24" s="7" t="s">
         <v>12</v>
@@ -1897,28 +1974,27 @@
         <v>9</v>
       </c>
       <c r="E24" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="F24" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="G24" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="H24" s="20" t="s">
         <v>90</v>
       </c>
-      <c r="F24" s="19" t="s">
-        <v>93</v>
-      </c>
-      <c r="G24" s="19" t="s">
-        <v>77</v>
-      </c>
-      <c r="H24" s="21" t="s">
-        <v>92</v>
-      </c>
       <c r="I24" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="J24" s="18" t="s">
-        <v>74</v>
+        <v>89</v>
+      </c>
+      <c r="J24" s="17" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="90" x14ac:dyDescent="0.25">
-      <c r="A25" s="6">
-        <f t="shared" si="0"/>
-        <v>20</v>
+      <c r="A25" s="6" t="s">
+        <v>173</v>
       </c>
       <c r="B25" s="7" t="s">
         <v>12</v>
@@ -1926,92 +2002,89 @@
       <c r="C25" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D25" s="22" t="s">
+      <c r="D25" s="21" t="s">
         <v>9</v>
       </c>
       <c r="E25" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="F25" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="G25" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="H25" s="20" t="s">
+        <v>94</v>
+      </c>
+      <c r="I25" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="F25" s="19" t="s">
-        <v>76</v>
-      </c>
-      <c r="G25" s="19" t="s">
-        <v>77</v>
-      </c>
-      <c r="H25" s="21" t="s">
+    </row>
+    <row r="26" spans="1:10" ht="120" x14ac:dyDescent="0.25">
+      <c r="A26" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="B26" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="C26" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D26" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="F26" s="18" t="s">
+        <v>97</v>
+      </c>
+      <c r="G26" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="H26" s="22" t="s">
         <v>96</v>
       </c>
-      <c r="I25" s="2" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" ht="120" x14ac:dyDescent="0.25">
-      <c r="A26" s="6">
-        <f t="shared" si="0"/>
-        <v>21</v>
-      </c>
-      <c r="B26" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="C26" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D26" s="22" t="s">
-        <v>9</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="F26" s="19" t="s">
-        <v>99</v>
-      </c>
-      <c r="G26" s="19" t="s">
+      <c r="I26" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="J26" s="20" t="s">
         <v>101</v>
       </c>
-      <c r="H26" s="23" t="s">
-        <v>98</v>
-      </c>
-      <c r="I26" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="J26" s="21" t="s">
+    </row>
+    <row r="27" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A27" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D27" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="F27" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="G27" s="18" t="s">
+        <v>84</v>
+      </c>
+      <c r="H27" s="22" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="27" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A27" s="6">
-        <f t="shared" si="0"/>
-        <v>22</v>
-      </c>
-      <c r="B27" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="C27" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D27" s="22" t="s">
-        <v>9</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="F27" s="19" t="s">
-        <v>76</v>
-      </c>
-      <c r="G27" s="19" t="s">
-        <v>86</v>
-      </c>
-      <c r="H27" s="23" t="s">
-        <v>105</v>
-      </c>
       <c r="I27" s="2" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="33" x14ac:dyDescent="0.25">
-      <c r="A28" s="6">
-        <f t="shared" si="0"/>
-        <v>23</v>
+      <c r="A28" s="6" t="s">
+        <v>176</v>
       </c>
       <c r="B28" s="7" t="s">
         <v>12</v>
@@ -2019,29 +2092,28 @@
       <c r="C28" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D28" s="22" t="s">
+      <c r="D28" s="21" t="s">
         <v>9</v>
       </c>
       <c r="E28" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="F28" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="G28" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="H28" s="19" t="s">
         <v>108</v>
       </c>
-      <c r="F28" s="19" t="s">
-        <v>70</v>
-      </c>
-      <c r="G28" s="19" t="s">
-        <v>77</v>
-      </c>
-      <c r="H28" s="20" t="s">
-        <v>110</v>
-      </c>
       <c r="I28" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="29" spans="1:10" ht="180" x14ac:dyDescent="0.25">
-      <c r="A29" s="6">
-        <f t="shared" si="0"/>
-        <v>24</v>
+      <c r="A29" s="6" t="s">
+        <v>175</v>
       </c>
       <c r="B29" s="7" t="s">
         <v>12</v>
@@ -2049,32 +2121,31 @@
       <c r="C29" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D29" s="22" t="s">
+      <c r="D29" s="21" t="s">
         <v>9</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="F29" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="G29" s="19" t="s">
-        <v>77</v>
-      </c>
-      <c r="H29" s="23" t="s">
+      <c r="F29" s="18" t="s">
+        <v>110</v>
+      </c>
+      <c r="G29" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="H29" s="22" t="s">
+        <v>109</v>
+      </c>
+      <c r="I29" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="I29" s="2" t="s">
+      <c r="J29" s="22" t="s">
         <v>113</v>
       </c>
-      <c r="J29" s="23" t="s">
-        <v>115</v>
-      </c>
     </row>
     <row r="30" spans="1:10" ht="180" x14ac:dyDescent="0.25">
-      <c r="A30" s="6">
-        <f t="shared" si="0"/>
-        <v>25</v>
+      <c r="A30" s="6" t="s">
+        <v>178</v>
       </c>
       <c r="B30" s="7" t="s">
         <v>12</v>
@@ -2082,32 +2153,31 @@
       <c r="C30" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D30" s="22" t="s">
+      <c r="D30" s="21" t="s">
         <v>9</v>
       </c>
       <c r="E30" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="F30" s="18" t="s">
+        <v>116</v>
+      </c>
+      <c r="G30" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="H30" s="19" t="s">
+        <v>114</v>
+      </c>
+      <c r="I30" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="F30" s="19" t="s">
-        <v>118</v>
-      </c>
-      <c r="G30" s="19" t="s">
-        <v>77</v>
-      </c>
-      <c r="H30" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="I30" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="J30" s="25" t="s">
-        <v>115</v>
+      <c r="J30" s="24" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="165" x14ac:dyDescent="0.25">
-      <c r="A31" s="6">
-        <f t="shared" si="0"/>
-        <v>26</v>
+      <c r="A31" s="6" t="s">
+        <v>179</v>
       </c>
       <c r="B31" s="7" t="s">
         <v>12</v>
@@ -2115,32 +2185,31 @@
       <c r="C31" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D31" s="22" t="s">
+      <c r="D31" s="21" t="s">
         <v>9</v>
       </c>
       <c r="E31" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F31" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="G31" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="H31" s="22" t="s">
+        <v>119</v>
+      </c>
+      <c r="I31" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="F31" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="G31" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="H31" s="23" t="s">
+      <c r="J31" s="22" t="s">
         <v>121</v>
       </c>
-      <c r="I31" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="J31" s="23" t="s">
-        <v>123</v>
-      </c>
     </row>
     <row r="32" spans="1:10" ht="195" x14ac:dyDescent="0.25">
-      <c r="A32" s="6">
-        <f t="shared" si="0"/>
-        <v>27</v>
+      <c r="A32" s="6" t="s">
+        <v>180</v>
       </c>
       <c r="B32" s="7" t="s">
         <v>12</v>
@@ -2148,32 +2217,31 @@
       <c r="C32" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D32" s="22" t="s">
+      <c r="D32" s="21" t="s">
         <v>9</v>
       </c>
       <c r="E32" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="F32" s="18" t="s">
+        <v>97</v>
+      </c>
+      <c r="G32" s="18" t="s">
+        <v>126</v>
+      </c>
+      <c r="H32" s="22" t="s">
+        <v>122</v>
+      </c>
+      <c r="I32" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="J32" s="22" t="s">
         <v>125</v>
       </c>
-      <c r="F32" s="19" t="s">
-        <v>99</v>
-      </c>
-      <c r="G32" s="19" t="s">
-        <v>128</v>
-      </c>
-      <c r="H32" s="23" t="s">
-        <v>124</v>
-      </c>
-      <c r="I32" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="J32" s="23" t="s">
-        <v>127</v>
-      </c>
     </row>
     <row r="33" spans="1:10" ht="165" x14ac:dyDescent="0.25">
-      <c r="A33" s="6">
-        <f t="shared" si="0"/>
-        <v>28</v>
+      <c r="A33" s="6" t="s">
+        <v>181</v>
       </c>
       <c r="B33" s="7" t="s">
         <v>12</v>
@@ -2181,65 +2249,63 @@
       <c r="C33" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D33" s="22" t="s">
+      <c r="D33" s="21" t="s">
         <v>9</v>
       </c>
       <c r="E33" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="F33" s="18" t="s">
+        <v>128</v>
+      </c>
+      <c r="G33" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="H33" s="22" t="s">
+        <v>127</v>
+      </c>
+      <c r="I33" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="J33" s="22" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="285" x14ac:dyDescent="0.25">
+      <c r="A34" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="B34" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="C34" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D34" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="E34" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="F33" s="19" t="s">
-        <v>130</v>
-      </c>
-      <c r="G33" s="19" t="s">
-        <v>77</v>
-      </c>
-      <c r="H33" s="23" t="s">
-        <v>129</v>
-      </c>
-      <c r="I33" s="2" t="s">
+      <c r="F34" s="18" t="s">
+        <v>134</v>
+      </c>
+      <c r="G34" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="H34" s="22" t="s">
+        <v>133</v>
+      </c>
+      <c r="I34" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="J33" s="23" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" ht="285" x14ac:dyDescent="0.25">
-      <c r="A34" s="6">
-        <f t="shared" si="0"/>
-        <v>29</v>
-      </c>
-      <c r="B34" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="C34" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D34" s="22" t="s">
-        <v>9</v>
-      </c>
-      <c r="E34" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="F34" s="19" t="s">
-        <v>136</v>
-      </c>
-      <c r="G34" s="19" t="s">
-        <v>77</v>
-      </c>
-      <c r="H34" s="23" t="s">
+      <c r="J34" s="22" t="s">
         <v>135</v>
       </c>
-      <c r="I34" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="J34" s="23" t="s">
-        <v>137</v>
-      </c>
     </row>
     <row r="35" spans="1:10" ht="180" x14ac:dyDescent="0.25">
-      <c r="A35" s="6">
-        <f t="shared" si="0"/>
-        <v>30</v>
+      <c r="A35" s="6" t="s">
+        <v>183</v>
       </c>
       <c r="B35" s="7" t="s">
         <v>12</v>
@@ -2247,32 +2313,31 @@
       <c r="C35" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D35" s="22" t="s">
+      <c r="D35" s="21" t="s">
         <v>9</v>
       </c>
       <c r="E35" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="F35" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="G35" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="H35" s="22" t="s">
         <v>138</v>
       </c>
-      <c r="F35" s="19" t="s">
-        <v>94</v>
-      </c>
-      <c r="G35" s="19" t="s">
-        <v>77</v>
-      </c>
-      <c r="H35" s="23" t="s">
-        <v>140</v>
-      </c>
       <c r="I35" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="J35" s="23" t="s">
+        <v>137</v>
+      </c>
+      <c r="J35" s="22" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="36" spans="1:10" ht="150" x14ac:dyDescent="0.25">
-      <c r="A36" s="6">
-        <f t="shared" si="0"/>
-        <v>31</v>
+      <c r="A36" s="6" t="s">
+        <v>184</v>
       </c>
       <c r="B36" s="7" t="s">
         <v>12</v>
@@ -2280,105 +2345,103 @@
       <c r="C36" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D36" s="22" t="s">
+      <c r="D36" s="21" t="s">
         <v>9</v>
       </c>
       <c r="E36" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="F36" s="18" t="s">
+        <v>142</v>
+      </c>
+      <c r="G36" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="H36" s="22" t="s">
+        <v>140</v>
+      </c>
+      <c r="I36" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="F36" s="19" t="s">
+      <c r="J36" s="22" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" ht="240" x14ac:dyDescent="0.25">
+      <c r="A37" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="B37" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D37" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="F37" s="18" t="s">
+        <v>97</v>
+      </c>
+      <c r="G37" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="H37" s="23" t="s">
+        <v>145</v>
+      </c>
+      <c r="I37" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="G36" s="19" t="s">
-        <v>77</v>
-      </c>
-      <c r="H36" s="23" t="s">
-        <v>142</v>
-      </c>
-      <c r="I36" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="J36" s="23" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" ht="240" x14ac:dyDescent="0.25">
-      <c r="A37" s="6">
-        <f t="shared" si="0"/>
-        <v>32</v>
-      </c>
-      <c r="B37" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="C37" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D37" s="22" t="s">
-        <v>9</v>
-      </c>
-      <c r="E37" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="F37" s="19" t="s">
+      <c r="J37" s="22" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" ht="180" x14ac:dyDescent="0.25">
+      <c r="A38" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="B38" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="C38" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D38" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="F38" s="18" t="s">
+        <v>149</v>
+      </c>
+      <c r="G38" s="18" t="s">
         <v>99</v>
       </c>
-      <c r="G37" s="19" t="s">
-        <v>77</v>
-      </c>
-      <c r="H37" s="24" t="s">
+      <c r="H38" s="19" t="s">
         <v>147</v>
       </c>
-      <c r="I37" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="J37" s="23" t="s">
+      <c r="I38" s="28" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="38" spans="1:10" ht="180" x14ac:dyDescent="0.25">
-      <c r="A38" s="6">
-        <f t="shared" si="0"/>
-        <v>33</v>
-      </c>
-      <c r="B38" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="C38" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D38" s="22" t="s">
-        <v>9</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="F38" s="19" t="s">
-        <v>151</v>
-      </c>
-      <c r="G38" s="19" t="s">
-        <v>101</v>
-      </c>
-      <c r="H38" s="20" t="s">
-        <v>149</v>
-      </c>
-      <c r="I38" s="19" t="s">
-        <v>150</v>
-      </c>
-      <c r="J38" s="23" t="s">
-        <v>115</v>
+      <c r="J38" s="22" t="s">
+        <v>113</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A5:J21" xr:uid="{00000000-0009-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A6:J21">
-      <sortCondition ref="A5:A21"/>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A6:J38">
+      <sortCondition descending="1" ref="A5:A21"/>
     </sortState>
   </autoFilter>
   <mergeCells count="2">
     <mergeCell ref="A4:XFD4"/>
     <mergeCell ref="A1:XFD3"/>
   </mergeCells>
-  <phoneticPr fontId="16" type="noConversion"/>
+  <phoneticPr fontId="15" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="E6" r:id="rId1" xr:uid="{96FE88B3-9B1A-4942-9E76-31B14B672BCB}"/>
     <hyperlink ref="I6" r:id="rId2" xr:uid="{076BC25F-DC3D-42A9-BC76-5B1D9BE1A295}"/>
@@ -2434,12 +2497,16 @@
     <hyperlink ref="E37" r:id="rId52" xr:uid="{E2145E7C-3713-40E3-84CA-74F81E34F1E8}"/>
     <hyperlink ref="I37" r:id="rId53" xr:uid="{6CB26260-4DAA-4CFE-8AAC-505327AED25F}"/>
     <hyperlink ref="E38" r:id="rId54" xr:uid="{3CC922C1-27F5-4E54-A1F6-A82FB93A2054}"/>
+    <hyperlink ref="I9" r:id="rId55" xr:uid="{AC844DC4-468A-47BC-8C3E-C235A0A0D1DB}"/>
+    <hyperlink ref="I12" r:id="rId56" xr:uid="{7595C12F-6479-472E-A71B-E8ED7C2C1DFF}"/>
+    <hyperlink ref="I13" r:id="rId57" xr:uid="{3C302E7B-FDFE-4FA1-84E4-693100362B35}"/>
+    <hyperlink ref="I38" r:id="rId58" xr:uid="{771EE190-08A0-4F64-A155-544FD55EEE7B}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" scale="41" fitToHeight="0" orientation="landscape" r:id="rId55"/>
+  <pageSetup paperSize="9" scale="41" fitToHeight="0" orientation="landscape" r:id="rId59"/>
   <headerFooter>
     <oddHeader>&amp;CPágina &amp;P</oddHeader>
   </headerFooter>
-  <drawing r:id="rId56"/>
+  <drawing r:id="rId60"/>
 </worksheet>
 </file>
</xml_diff>